<commit_message>
fix: dashboard corrigido - eixos, labels, horas 1 decimal, % inteiro, sem simulacao
</commit_message>
<xml_diff>
--- a/Relacao_Pv.xlsx
+++ b/Relacao_Pv.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA515174-255C-4808-A430-DBE895D87288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B5F714-A92D-46FB-B7E8-12FDB07057C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A0122E1E-44D4-425A-97B9-4BCE5080F7F6}"/>
+    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{A0122E1E-44D4-425A-97B9-4BCE5080F7F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
atualizacao banco de dados de planilhas excel
</commit_message>
<xml_diff>
--- a/Relacao_Pv.xlsx
+++ b/Relacao_Pv.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09CDC72F-570E-4843-A4B6-F74A4599886A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9B20FD-49E4-46EE-80D3-528EB99AC313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,37 +16,16 @@
     <sheet name="ItensPedidosVenda" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ItensPedidosVenda!$A$1:$E$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ItensPedidosVenda!$A$1:$E$185</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="49">
   <si>
     <t>MAGVATECH</t>
-  </si>
-  <si>
-    <t>B13AMY11112</t>
-  </si>
-  <si>
-    <t>B13AN511113</t>
-  </si>
-  <si>
-    <t>B13AN511112</t>
-  </si>
-  <si>
-    <t>B13AMN11112</t>
-  </si>
-  <si>
-    <t>B13AMG11112</t>
-  </si>
-  <si>
-    <t>B13AMG11113</t>
-  </si>
-  <si>
-    <t>B13AN311112</t>
   </si>
   <si>
     <t>GE - RBH</t>
@@ -1001,7 +980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E185"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
@@ -1013,30 +992,30 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>6552</v>
+        <v>6549</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1">
         <v>46113</v>
@@ -1047,13 +1026,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>6549</v>
+        <v>6552</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1">
         <v>46113</v>
@@ -1067,10 +1046,10 @@
         <v>6764</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1">
         <v>46113</v>
@@ -1084,10 +1063,10 @@
         <v>6780</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D5" s="1">
         <v>46113</v>
@@ -1101,10 +1080,10 @@
         <v>6873</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D6" s="1">
         <v>46113</v>
@@ -1115,13 +1094,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>6553</v>
+        <v>6550</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D7" s="1">
         <v>46118</v>
@@ -1132,13 +1111,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>6550</v>
+        <v>6553</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D8" s="1">
         <v>46118</v>
@@ -1149,36 +1128,36 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>6710</v>
+        <v>6696</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>15967961</v>
       </c>
       <c r="D9" s="1">
         <v>46118</v>
       </c>
       <c r="E9">
-        <v>146</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>6696</v>
+        <v>6710</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10">
-        <v>15967961</v>
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
       </c>
       <c r="D10" s="1">
         <v>46118</v>
       </c>
       <c r="E10">
-        <v>102</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1186,7 +1165,7 @@
         <v>6734</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C11">
         <v>14558705</v>
@@ -1200,121 +1179,121 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>6762</v>
+        <v>6756</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C12">
-        <v>12421834</v>
+        <v>13991667</v>
       </c>
       <c r="D12" s="1">
         <v>46118</v>
       </c>
       <c r="E12">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>6761</v>
+        <v>6757</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C13">
-        <v>13319685</v>
+        <v>13991819</v>
       </c>
       <c r="D13" s="1">
         <v>46118</v>
       </c>
       <c r="E13">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>6760</v>
+        <v>6758</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C14">
-        <v>11469602</v>
+        <v>13991818</v>
       </c>
       <c r="D14" s="1">
         <v>46118</v>
       </c>
       <c r="E14">
-        <v>48</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>6758</v>
+        <v>6760</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C15">
-        <v>13991818</v>
+        <v>11469602</v>
       </c>
       <c r="D15" s="1">
         <v>46118</v>
       </c>
       <c r="E15">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>6757</v>
+        <v>6761</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C16">
-        <v>13991819</v>
+        <v>13319685</v>
       </c>
       <c r="D16" s="1">
         <v>46118</v>
       </c>
       <c r="E16">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>6756</v>
+        <v>6762</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C17">
-        <v>13991667</v>
+        <v>12421834</v>
       </c>
       <c r="D17" s="1">
         <v>46118</v>
       </c>
       <c r="E17">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>6773</v>
+        <v>6771</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C18">
-        <v>14140591</v>
+        <v>15976733</v>
       </c>
       <c r="D18" s="1">
         <v>46118</v>
       </c>
       <c r="E18">
-        <v>30</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1322,7 +1301,7 @@
         <v>6772</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C19">
         <v>15976244</v>
@@ -1336,30 +1315,30 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>6771</v>
+        <v>6773</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C20">
-        <v>15976733</v>
+        <v>14140591</v>
       </c>
       <c r="D20" s="1">
         <v>46118</v>
       </c>
       <c r="E20">
-        <v>87</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>6790</v>
+        <v>6789</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C21">
-        <v>13991663</v>
+        <v>13991909</v>
       </c>
       <c r="D21" s="1">
         <v>46118</v>
@@ -1370,13 +1349,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>6789</v>
+        <v>6790</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C22">
-        <v>13991909</v>
+        <v>13991663</v>
       </c>
       <c r="D22" s="1">
         <v>46118</v>
@@ -1387,53 +1366,53 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>6838</v>
+        <v>6832</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C23">
-        <v>11467111</v>
+        <v>13588930</v>
       </c>
       <c r="D23" s="1">
         <v>46118</v>
       </c>
       <c r="E23">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>6837</v>
+        <v>6833</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C24">
-        <v>11468114</v>
+        <v>14577954</v>
       </c>
       <c r="D24" s="1">
         <v>46118</v>
       </c>
       <c r="E24">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>6836</v>
+        <v>6834</v>
       </c>
       <c r="B25" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C25">
-        <v>11468775</v>
+        <v>14577949</v>
       </c>
       <c r="D25" s="1">
         <v>46118</v>
       </c>
       <c r="E25">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -1441,7 +1420,7 @@
         <v>6835</v>
       </c>
       <c r="B26" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C26">
         <v>11468826</v>
@@ -1455,53 +1434,53 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>6834</v>
+        <v>6836</v>
       </c>
       <c r="B27" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C27">
-        <v>14577949</v>
+        <v>11468775</v>
       </c>
       <c r="D27" s="1">
         <v>46118</v>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>6833</v>
+        <v>6837</v>
       </c>
       <c r="B28" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C28">
-        <v>14577954</v>
+        <v>11468114</v>
       </c>
       <c r="D28" s="1">
         <v>46118</v>
       </c>
       <c r="E28">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>6832</v>
+        <v>6838</v>
       </c>
       <c r="B29" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C29">
-        <v>13588930</v>
+        <v>11467111</v>
       </c>
       <c r="D29" s="1">
         <v>46118</v>
       </c>
       <c r="E29">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1509,10 +1488,10 @@
         <v>6842</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D30" s="1">
         <v>46119</v>
@@ -1526,10 +1505,10 @@
         <v>6859</v>
       </c>
       <c r="B31" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C31" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D31" s="1">
         <v>46120</v>
@@ -1543,10 +1522,10 @@
         <v>6519</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D32" s="1">
         <v>46121</v>
@@ -1557,36 +1536,36 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>6875</v>
+        <v>6870</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D33" s="1">
         <v>46121</v>
       </c>
       <c r="E33">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>6870</v>
+        <v>6875</v>
       </c>
       <c r="B34" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C34" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D34" s="1">
         <v>46121</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1594,10 +1573,10 @@
         <v>6953</v>
       </c>
       <c r="B35" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D35" s="1">
         <v>46121</v>
@@ -1608,376 +1587,376 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>3746</v>
+        <v>6013</v>
       </c>
       <c r="B36" t="s">
         <v>0</v>
       </c>
       <c r="C36" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="1">
         <v>46122</v>
       </c>
       <c r="E36">
-        <v>5</v>
+        <v>500</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>3746</v>
+        <v>6522</v>
       </c>
       <c r="B37" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D37" s="1">
         <v>46122</v>
       </c>
       <c r="E37">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>3746</v>
+        <v>6797</v>
       </c>
       <c r="B38" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C38" t="s">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="D38" s="1">
         <v>46122</v>
       </c>
       <c r="E38">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>3746</v>
+        <v>6798</v>
       </c>
       <c r="B39" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="D39" s="1">
         <v>46122</v>
       </c>
       <c r="E39">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>3746</v>
+        <v>6827</v>
       </c>
       <c r="B40" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D40" s="1">
         <v>46122</v>
       </c>
       <c r="E40">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>3746</v>
+        <v>6830</v>
       </c>
       <c r="B41" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D41" s="1">
         <v>46122</v>
       </c>
       <c r="E41">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>3746</v>
+        <v>6754</v>
       </c>
       <c r="B42" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="1">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="E42">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>6013</v>
+        <v>6942</v>
       </c>
       <c r="B43" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D43" s="1">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="E43">
-        <v>200</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>6013</v>
+        <v>6712</v>
       </c>
       <c r="B44" t="s">
-        <v>0</v>
-      </c>
-      <c r="C44" t="s">
-        <v>9</v>
+        <v>15</v>
+      </c>
+      <c r="C44">
+        <v>15970137</v>
       </c>
       <c r="D44" s="1">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="E44">
-        <v>150</v>
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>6013</v>
+        <v>6774</v>
       </c>
       <c r="B45" t="s">
-        <v>0</v>
-      </c>
-      <c r="C45" t="s">
-        <v>9</v>
+        <v>15</v>
+      </c>
+      <c r="C45">
+        <v>14153893</v>
       </c>
       <c r="D45" s="1">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="E45">
-        <v>150</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>6522</v>
+        <v>6821</v>
       </c>
       <c r="B46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46">
+        <v>14085079</v>
+      </c>
+      <c r="D46" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E46">
         <v>12</v>
-      </c>
-      <c r="C46" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="1">
-        <v>46122</v>
-      </c>
-      <c r="E46">
-        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>6798</v>
+        <v>6847</v>
       </c>
       <c r="B47" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47">
+        <v>14627922</v>
+      </c>
+      <c r="D47" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E47">
         <v>12</v>
-      </c>
-      <c r="C47" t="s">
-        <v>34</v>
-      </c>
-      <c r="D47" s="1">
-        <v>46122</v>
-      </c>
-      <c r="E47">
-        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>6797</v>
+        <v>6848</v>
       </c>
       <c r="B48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C48" t="s">
-        <v>34</v>
+        <v>15</v>
+      </c>
+      <c r="C48">
+        <v>14035990</v>
       </c>
       <c r="D48" s="1">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>6827</v>
+        <v>6849</v>
       </c>
       <c r="B49" t="s">
-        <v>12</v>
-      </c>
-      <c r="C49" t="s">
-        <v>32</v>
+        <v>15</v>
+      </c>
+      <c r="C49">
+        <v>14624464</v>
       </c>
       <c r="D49" s="1">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>6830</v>
+        <v>6850</v>
       </c>
       <c r="B50" t="s">
-        <v>12</v>
-      </c>
-      <c r="C50" t="s">
-        <v>36</v>
+        <v>15</v>
+      </c>
+      <c r="C50">
+        <v>14613011</v>
       </c>
       <c r="D50" s="1">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="E50">
-        <v>10</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>6754</v>
+        <v>6851</v>
       </c>
       <c r="B51" t="s">
-        <v>12</v>
-      </c>
-      <c r="C51" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="C51">
+        <v>11510278</v>
       </c>
       <c r="D51" s="1">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="E51">
-        <v>7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>6942</v>
+        <v>6852</v>
       </c>
       <c r="B52" t="s">
-        <v>8</v>
-      </c>
-      <c r="C52" t="s">
-        <v>30</v>
+        <v>15</v>
+      </c>
+      <c r="C52">
+        <v>15975246</v>
       </c>
       <c r="D52" s="1">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>54</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>6712</v>
+        <v>6853</v>
       </c>
       <c r="B53" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C53">
-        <v>15970137</v>
+        <v>15973874</v>
       </c>
       <c r="D53" s="1">
         <v>46125</v>
       </c>
       <c r="E53">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>6774</v>
+        <v>6854</v>
       </c>
       <c r="B54" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C54">
-        <v>14153893</v>
+        <v>15972626</v>
       </c>
       <c r="D54" s="1">
         <v>46125</v>
       </c>
       <c r="E54">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>6821</v>
+        <v>6855</v>
       </c>
       <c r="B55" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C55">
-        <v>14085079</v>
+        <v>15972619</v>
       </c>
       <c r="D55" s="1">
         <v>46125</v>
       </c>
       <c r="E55">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>6861</v>
+        <v>6856</v>
       </c>
       <c r="B56" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C56">
-        <v>14084370</v>
+        <v>15972293</v>
       </c>
       <c r="D56" s="1">
         <v>46125</v>
       </c>
       <c r="E56">
-        <v>12</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>6860</v>
+        <v>6857</v>
       </c>
       <c r="B57" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C57">
-        <v>14095131</v>
+        <v>15972104</v>
       </c>
       <c r="D57" s="1">
         <v>46125</v>
       </c>
       <c r="E57">
-        <v>12</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
@@ -1985,7 +1964,7 @@
         <v>6858</v>
       </c>
       <c r="B58" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C58">
         <v>15971930</v>
@@ -1999,200 +1978,200 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>6857</v>
+        <v>6860</v>
       </c>
       <c r="B59" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C59">
-        <v>15972104</v>
+        <v>14095131</v>
       </c>
       <c r="D59" s="1">
         <v>46125</v>
       </c>
       <c r="E59">
-        <v>54</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>6856</v>
+        <v>6861</v>
       </c>
       <c r="B60" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C60">
-        <v>15972293</v>
+        <v>14084370</v>
       </c>
       <c r="D60" s="1">
         <v>46125</v>
       </c>
       <c r="E60">
-        <v>54</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>6855</v>
+        <v>6862</v>
       </c>
       <c r="B61" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C61">
-        <v>15972619</v>
+        <v>15790045</v>
       </c>
       <c r="D61" s="1">
         <v>46125</v>
       </c>
       <c r="E61">
-        <v>27</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>6854</v>
+        <v>6863</v>
       </c>
       <c r="B62" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C62">
-        <v>15972626</v>
+        <v>15790121</v>
       </c>
       <c r="D62" s="1">
         <v>46125</v>
       </c>
       <c r="E62">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>6853</v>
+        <v>6864</v>
       </c>
       <c r="B63" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C63">
-        <v>15973874</v>
+        <v>15790046</v>
       </c>
       <c r="D63" s="1">
         <v>46125</v>
       </c>
       <c r="E63">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>6852</v>
+        <v>6865</v>
       </c>
       <c r="B64" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C64">
-        <v>15975246</v>
+        <v>14563966</v>
       </c>
       <c r="D64" s="1">
         <v>46125</v>
       </c>
       <c r="E64">
-        <v>54</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>6851</v>
+        <v>6866</v>
       </c>
       <c r="B65" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C65">
-        <v>11510278</v>
+        <v>14563925</v>
       </c>
       <c r="D65" s="1">
         <v>46125</v>
       </c>
       <c r="E65">
-        <v>100</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>6850</v>
+        <v>6867</v>
       </c>
       <c r="B66" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C66">
-        <v>14613011</v>
+        <v>15540457</v>
       </c>
       <c r="D66" s="1">
         <v>46125</v>
       </c>
       <c r="E66">
-        <v>48</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>6849</v>
+        <v>6868</v>
       </c>
       <c r="B67" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C67">
-        <v>14624464</v>
+        <v>15540450</v>
       </c>
       <c r="D67" s="1">
         <v>46125</v>
       </c>
       <c r="E67">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>6848</v>
+        <v>6869</v>
       </c>
       <c r="B68" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C68">
-        <v>14035990</v>
+        <v>15494648</v>
       </c>
       <c r="D68" s="1">
         <v>46125</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>6847</v>
+        <v>6895</v>
       </c>
       <c r="B69" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C69">
-        <v>14627922</v>
+        <v>11463275</v>
       </c>
       <c r="D69" s="1">
         <v>46125</v>
       </c>
       <c r="E69">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>6869</v>
+        <v>6896</v>
       </c>
       <c r="B70" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C70">
-        <v>15494648</v>
+        <v>11463274</v>
       </c>
       <c r="D70" s="1">
         <v>46125</v>
@@ -2203,13 +2182,13 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>6868</v>
+        <v>6897</v>
       </c>
       <c r="B71" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C71">
-        <v>15540450</v>
+        <v>11460670</v>
       </c>
       <c r="D71" s="1">
         <v>46125</v>
@@ -2220,13 +2199,13 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>6867</v>
+        <v>6898</v>
       </c>
       <c r="B72" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C72">
-        <v>15540457</v>
+        <v>11458375</v>
       </c>
       <c r="D72" s="1">
         <v>46125</v>
@@ -2237,13 +2216,13 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>6866</v>
+        <v>6899</v>
       </c>
       <c r="B73" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C73">
-        <v>14563925</v>
+        <v>11460314</v>
       </c>
       <c r="D73" s="1">
         <v>46125</v>
@@ -2254,13 +2233,13 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>6865</v>
+        <v>6900</v>
       </c>
       <c r="B74" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C74">
-        <v>14563966</v>
+        <v>13833429</v>
       </c>
       <c r="D74" s="1">
         <v>46125</v>
@@ -2271,353 +2250,353 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75">
-        <v>6864</v>
+        <v>6909</v>
       </c>
       <c r="B75" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C75">
-        <v>15790046</v>
+        <v>11510278</v>
       </c>
       <c r="D75" s="1">
         <v>46125</v>
       </c>
       <c r="E75">
-        <v>3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>6863</v>
+        <v>6767</v>
       </c>
       <c r="B76" t="s">
-        <v>22</v>
-      </c>
-      <c r="C76">
-        <v>15790121</v>
+        <v>5</v>
+      </c>
+      <c r="C76" t="s">
+        <v>11</v>
       </c>
       <c r="D76" s="1">
-        <v>46125</v>
+        <v>46127</v>
       </c>
       <c r="E76">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>6862</v>
+        <v>6770</v>
       </c>
       <c r="B77" t="s">
-        <v>22</v>
-      </c>
-      <c r="C77">
-        <v>15790045</v>
+        <v>5</v>
+      </c>
+      <c r="C77" t="s">
+        <v>17</v>
       </c>
       <c r="D77" s="1">
-        <v>46125</v>
+        <v>46127</v>
       </c>
       <c r="E77">
-        <v>6</v>
+        <v>62</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>6909</v>
+        <v>6828</v>
       </c>
       <c r="B78" t="s">
-        <v>22</v>
-      </c>
-      <c r="C78">
-        <v>11510278</v>
+        <v>5</v>
+      </c>
+      <c r="C78" t="s">
+        <v>10</v>
       </c>
       <c r="D78" s="1">
-        <v>46125</v>
+        <v>46127</v>
       </c>
       <c r="E78">
-        <v>100</v>
+        <v>51</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>6900</v>
+        <v>6547</v>
       </c>
       <c r="B79" t="s">
-        <v>22</v>
-      </c>
-      <c r="C79">
-        <v>13833429</v>
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>4</v>
       </c>
       <c r="D79" s="1">
-        <v>46125</v>
+        <v>46128</v>
       </c>
       <c r="E79">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>6899</v>
+        <v>6554</v>
       </c>
       <c r="B80" t="s">
-        <v>22</v>
-      </c>
-      <c r="C80">
-        <v>11460314</v>
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>3</v>
       </c>
       <c r="D80" s="1">
-        <v>46125</v>
+        <v>46128</v>
       </c>
       <c r="E80">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81">
-        <v>6898</v>
+        <v>6814</v>
       </c>
       <c r="B81" t="s">
-        <v>22</v>
-      </c>
-      <c r="C81">
-        <v>11458375</v>
+        <v>5</v>
+      </c>
+      <c r="C81" t="s">
+        <v>28</v>
       </c>
       <c r="D81" s="1">
-        <v>46125</v>
+        <v>46129</v>
       </c>
       <c r="E81">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82">
-        <v>6897</v>
+        <v>6713</v>
       </c>
       <c r="B82" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C82">
-        <v>11460670</v>
+        <v>15970137</v>
       </c>
       <c r="D82" s="1">
-        <v>46125</v>
+        <v>46132</v>
       </c>
       <c r="E82">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>6896</v>
+        <v>6727</v>
       </c>
       <c r="B83" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C83">
-        <v>11463274</v>
+        <v>15967961</v>
       </c>
       <c r="D83" s="1">
-        <v>46125</v>
+        <v>46132</v>
       </c>
       <c r="E83">
-        <v>6</v>
+        <v>123</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>6895</v>
+        <v>6788</v>
       </c>
       <c r="B84" t="s">
-        <v>22</v>
-      </c>
-      <c r="C84">
-        <v>11463275</v>
+        <v>5</v>
+      </c>
+      <c r="C84" t="s">
+        <v>19</v>
       </c>
       <c r="D84" s="1">
-        <v>46125</v>
+        <v>46132</v>
       </c>
       <c r="E84">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>6770</v>
+        <v>6793</v>
       </c>
       <c r="B85" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C85" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D85" s="1">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="E85">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86">
-        <v>6767</v>
+        <v>6799</v>
       </c>
       <c r="B86" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C86" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D86" s="1">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>6828</v>
+        <v>6819</v>
       </c>
       <c r="B87" t="s">
-        <v>12</v>
-      </c>
-      <c r="C87" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="C87">
+        <v>11893661</v>
       </c>
       <c r="D87" s="1">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="E87">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88">
-        <v>6554</v>
+        <v>6822</v>
       </c>
       <c r="B88" t="s">
-        <v>8</v>
-      </c>
-      <c r="C88" t="s">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="C88">
+        <v>14496774</v>
       </c>
       <c r="D88" s="1">
-        <v>46128</v>
+        <v>46132</v>
       </c>
       <c r="E88">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89">
-        <v>6547</v>
+        <v>6823</v>
       </c>
       <c r="B89" t="s">
-        <v>8</v>
-      </c>
-      <c r="C89" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="C89">
+        <v>17800490</v>
       </c>
       <c r="D89" s="1">
-        <v>46128</v>
+        <v>46132</v>
       </c>
       <c r="E89">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90">
-        <v>6814</v>
+        <v>6824</v>
       </c>
       <c r="B90" t="s">
-        <v>12</v>
-      </c>
-      <c r="C90" t="s">
-        <v>35</v>
+        <v>15</v>
+      </c>
+      <c r="C90">
+        <v>14504560</v>
       </c>
       <c r="D90" s="1">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="E90">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91">
-        <v>6713</v>
+        <v>6825</v>
       </c>
       <c r="B91" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C91">
-        <v>15970137</v>
+        <v>17797436</v>
       </c>
       <c r="D91" s="1">
         <v>46132</v>
       </c>
       <c r="E91">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92">
-        <v>6727</v>
+        <v>6846</v>
       </c>
       <c r="B92" t="s">
-        <v>22</v>
-      </c>
-      <c r="C92">
-        <v>15967961</v>
+        <v>5</v>
+      </c>
+      <c r="C92" t="s">
+        <v>13</v>
       </c>
       <c r="D92" s="1">
         <v>46132</v>
       </c>
       <c r="E92">
-        <v>123</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93">
-        <v>6788</v>
+        <v>6893</v>
       </c>
       <c r="B93" t="s">
-        <v>12</v>
-      </c>
-      <c r="C93" t="s">
-        <v>26</v>
+        <v>15</v>
+      </c>
+      <c r="C93">
+        <v>13829680</v>
       </c>
       <c r="D93" s="1">
         <v>46132</v>
       </c>
       <c r="E93">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94">
-        <v>6793</v>
+        <v>6894</v>
       </c>
       <c r="B94" t="s">
-        <v>12</v>
-      </c>
-      <c r="C94" t="s">
-        <v>26</v>
+        <v>15</v>
+      </c>
+      <c r="C94">
+        <v>13592346</v>
       </c>
       <c r="D94" s="1">
         <v>46132</v>
       </c>
       <c r="E94">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95">
-        <v>6799</v>
+        <v>6901</v>
       </c>
       <c r="B95" t="s">
-        <v>12</v>
-      </c>
-      <c r="C95" t="s">
-        <v>33</v>
+        <v>15</v>
+      </c>
+      <c r="C95">
+        <v>15982393</v>
       </c>
       <c r="D95" s="1">
         <v>46132</v>
@@ -2628,13 +2607,13 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96">
-        <v>6825</v>
+        <v>6902</v>
       </c>
       <c r="B96" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C96">
-        <v>17797436</v>
+        <v>13828817</v>
       </c>
       <c r="D96" s="1">
         <v>46132</v>
@@ -2645,560 +2624,560 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97">
-        <v>6824</v>
+        <v>6911</v>
       </c>
       <c r="B97" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C97">
-        <v>14504560</v>
+        <v>16727617</v>
       </c>
       <c r="D97" s="1">
         <v>46132</v>
       </c>
       <c r="E97">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98">
-        <v>6823</v>
+        <v>6912</v>
       </c>
       <c r="B98" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C98">
-        <v>17800490</v>
+        <v>11440086</v>
       </c>
       <c r="D98" s="1">
         <v>46132</v>
       </c>
       <c r="E98">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99">
-        <v>6822</v>
+        <v>6913</v>
       </c>
       <c r="B99" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C99">
-        <v>14496774</v>
+        <v>13832165</v>
       </c>
       <c r="D99" s="1">
         <v>46132</v>
       </c>
       <c r="E99">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100">
-        <v>6819</v>
+        <v>6916</v>
       </c>
       <c r="B100" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C100">
-        <v>11893661</v>
+        <v>12420856</v>
       </c>
       <c r="D100" s="1">
         <v>46132</v>
       </c>
       <c r="E100">
-        <v>36</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101">
-        <v>6846</v>
+        <v>6917</v>
       </c>
       <c r="B101" t="s">
-        <v>12</v>
-      </c>
-      <c r="C101" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="C101">
+        <v>12420855</v>
       </c>
       <c r="D101" s="1">
         <v>46132</v>
       </c>
       <c r="E101">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102">
-        <v>6912</v>
+        <v>6918</v>
       </c>
       <c r="B102" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C102">
-        <v>11440086</v>
+        <v>12406511</v>
       </c>
       <c r="D102" s="1">
         <v>46132</v>
       </c>
       <c r="E102">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103">
-        <v>6911</v>
+        <v>6919</v>
       </c>
       <c r="B103" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C103">
-        <v>16727617</v>
+        <v>12406391</v>
       </c>
       <c r="D103" s="1">
         <v>46132</v>
       </c>
       <c r="E103">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104">
-        <v>6902</v>
+        <v>6920</v>
       </c>
       <c r="B104" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C104">
-        <v>13828817</v>
+        <v>16406069</v>
       </c>
       <c r="D104" s="1">
         <v>46132</v>
       </c>
       <c r="E104">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105">
-        <v>6901</v>
+        <v>6765</v>
       </c>
       <c r="B105" t="s">
-        <v>22</v>
-      </c>
-      <c r="C105">
-        <v>15982393</v>
+        <v>5</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
       </c>
       <c r="D105" s="1">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="E105">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106">
-        <v>6894</v>
+        <v>6839</v>
       </c>
       <c r="B106" t="s">
-        <v>22</v>
-      </c>
-      <c r="C106">
-        <v>13592346</v>
+        <v>5</v>
+      </c>
+      <c r="C106" t="s">
+        <v>28</v>
       </c>
       <c r="D106" s="1">
-        <v>46132</v>
+        <v>46134</v>
       </c>
       <c r="E106">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107">
-        <v>6893</v>
+        <v>6637</v>
       </c>
       <c r="B107" t="s">
-        <v>22</v>
-      </c>
-      <c r="C107">
-        <v>13829680</v>
+        <v>5</v>
+      </c>
+      <c r="C107" t="s">
+        <v>12</v>
       </c>
       <c r="D107" s="1">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="E107">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108">
-        <v>6920</v>
+        <v>6766</v>
       </c>
       <c r="B108" t="s">
-        <v>22</v>
-      </c>
-      <c r="C108">
-        <v>16406069</v>
+        <v>5</v>
+      </c>
+      <c r="C108" t="s">
+        <v>7</v>
       </c>
       <c r="D108" s="1">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="E108">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109">
-        <v>6919</v>
+        <v>6784</v>
       </c>
       <c r="B109" t="s">
-        <v>22</v>
-      </c>
-      <c r="C109">
-        <v>12406391</v>
+        <v>5</v>
+      </c>
+      <c r="C109" t="s">
+        <v>20</v>
       </c>
       <c r="D109" s="1">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="E109">
-        <v>6</v>
+        <v>200</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110">
-        <v>6918</v>
+        <v>6843</v>
       </c>
       <c r="B110" t="s">
-        <v>22</v>
-      </c>
-      <c r="C110">
-        <v>12406511</v>
+        <v>5</v>
+      </c>
+      <c r="C110" t="s">
+        <v>32</v>
       </c>
       <c r="D110" s="1">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="E110">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111">
-        <v>6917</v>
+        <v>6941</v>
       </c>
       <c r="B111" t="s">
-        <v>22</v>
-      </c>
-      <c r="C111">
-        <v>12420855</v>
+        <v>5</v>
+      </c>
+      <c r="C111" t="s">
+        <v>13</v>
       </c>
       <c r="D111" s="1">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="E111">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112">
-        <v>6916</v>
+        <v>6786</v>
       </c>
       <c r="B112" t="s">
-        <v>22</v>
-      </c>
-      <c r="C112">
-        <v>12420856</v>
+        <v>5</v>
+      </c>
+      <c r="C112" t="s">
+        <v>8</v>
       </c>
       <c r="D112" s="1">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="E112">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113">
-        <v>6913</v>
+        <v>6820</v>
       </c>
       <c r="B113" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C113">
-        <v>13832165</v>
+        <v>12864933</v>
       </c>
       <c r="D113" s="1">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="E113">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114">
-        <v>6765</v>
+        <v>6910</v>
       </c>
       <c r="B114" t="s">
-        <v>12</v>
-      </c>
-      <c r="C114" t="s">
-        <v>25</v>
+        <v>15</v>
+      </c>
+      <c r="C114">
+        <v>11510278</v>
       </c>
       <c r="D114" s="1">
-        <v>46133</v>
+        <v>46139</v>
       </c>
       <c r="E114">
-        <v>2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115">
-        <v>6839</v>
+        <v>6921</v>
       </c>
       <c r="B115" t="s">
-        <v>12</v>
-      </c>
-      <c r="C115" t="s">
-        <v>35</v>
+        <v>15</v>
+      </c>
+      <c r="C115">
+        <v>15494649</v>
       </c>
       <c r="D115" s="1">
-        <v>46134</v>
+        <v>46139</v>
       </c>
       <c r="E115">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116">
-        <v>6637</v>
+        <v>6922</v>
       </c>
       <c r="B116" t="s">
-        <v>12</v>
-      </c>
-      <c r="C116" t="s">
-        <v>19</v>
+        <v>15</v>
+      </c>
+      <c r="C116">
+        <v>14494848</v>
       </c>
       <c r="D116" s="1">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="E116">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117">
-        <v>6766</v>
+        <v>6923</v>
       </c>
       <c r="B117" t="s">
-        <v>12</v>
-      </c>
-      <c r="C117" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="C117">
+        <v>13279123</v>
       </c>
       <c r="D117" s="1">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="E117">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118">
-        <v>6784</v>
+        <v>6924</v>
       </c>
       <c r="B118" t="s">
-        <v>12</v>
-      </c>
-      <c r="C118" t="s">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="C118">
+        <v>13202650</v>
       </c>
       <c r="D118" s="1">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="E118">
-        <v>200</v>
+        <v>6</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119">
-        <v>6843</v>
+        <v>6925</v>
       </c>
       <c r="B119" t="s">
-        <v>12</v>
-      </c>
-      <c r="C119" t="s">
-        <v>39</v>
+        <v>15</v>
+      </c>
+      <c r="C119">
+        <v>13993039</v>
       </c>
       <c r="D119" s="1">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120">
-        <v>6941</v>
+        <v>6926</v>
       </c>
       <c r="B120" t="s">
+        <v>15</v>
+      </c>
+      <c r="C120">
+        <v>15481651</v>
+      </c>
+      <c r="D120" s="1">
+        <v>46139</v>
+      </c>
+      <c r="E120">
         <v>12</v>
-      </c>
-      <c r="C120" t="s">
-        <v>20</v>
-      </c>
-      <c r="D120" s="1">
-        <v>46135</v>
-      </c>
-      <c r="E120">
-        <v>1</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121">
-        <v>6786</v>
+        <v>6927</v>
       </c>
       <c r="B121" t="s">
-        <v>12</v>
-      </c>
-      <c r="C121" t="s">
-        <v>15</v>
+        <v>15</v>
+      </c>
+      <c r="C121">
+        <v>13319535</v>
       </c>
       <c r="D121" s="1">
         <v>46139</v>
       </c>
       <c r="E121">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122">
-        <v>6820</v>
+        <v>6640</v>
       </c>
       <c r="B122" t="s">
-        <v>22</v>
-      </c>
-      <c r="C122">
-        <v>12864933</v>
+        <v>5</v>
+      </c>
+      <c r="C122" t="s">
+        <v>9</v>
       </c>
       <c r="D122" s="1">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="E122">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123">
-        <v>6910</v>
+        <v>6641</v>
       </c>
       <c r="B123" t="s">
-        <v>22</v>
-      </c>
-      <c r="C123">
-        <v>11510278</v>
+        <v>5</v>
+      </c>
+      <c r="C123" t="s">
+        <v>6</v>
       </c>
       <c r="D123" s="1">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="E123">
-        <v>50</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124">
-        <v>6927</v>
+        <v>6885</v>
       </c>
       <c r="B124" t="s">
-        <v>22</v>
-      </c>
-      <c r="C124">
-        <v>13319535</v>
+        <v>5</v>
+      </c>
+      <c r="C124" t="s">
+        <v>41</v>
       </c>
       <c r="D124" s="1">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="E124">
-        <v>6</v>
+        <v>50</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125">
-        <v>6926</v>
+        <v>6831</v>
       </c>
       <c r="B125" t="s">
-        <v>22</v>
-      </c>
-      <c r="C125">
-        <v>15481651</v>
+        <v>5</v>
+      </c>
+      <c r="C125" t="s">
+        <v>24</v>
       </c>
       <c r="D125" s="1">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="E125">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126">
-        <v>6925</v>
+        <v>6903</v>
       </c>
       <c r="B126" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C126">
-        <v>13993039</v>
+        <v>13828817</v>
       </c>
       <c r="D126" s="1">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E126">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127">
-        <v>6924</v>
+        <v>6906</v>
       </c>
       <c r="B127" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C127">
-        <v>13202650</v>
+        <v>15967965</v>
       </c>
       <c r="D127" s="1">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E127">
-        <v>6</v>
+        <v>39</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128">
-        <v>6923</v>
+        <v>6914</v>
       </c>
       <c r="B128" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C128">
-        <v>13279123</v>
+        <v>13832165</v>
       </c>
       <c r="D128" s="1">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E128">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129">
-        <v>6922</v>
+        <v>6928</v>
       </c>
       <c r="B129" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C129">
-        <v>14494848</v>
+        <v>14085079</v>
       </c>
       <c r="D129" s="1">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E129">
         <v>6</v>
@@ -3206,526 +3185,526 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130">
-        <v>6921</v>
+        <v>6929</v>
       </c>
       <c r="B130" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C130">
-        <v>15494649</v>
+        <v>14153893</v>
       </c>
       <c r="D130" s="1">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E130">
-        <v>6</v>
+        <v>57</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131">
-        <v>6641</v>
+        <v>6930</v>
       </c>
       <c r="B131" t="s">
-        <v>12</v>
-      </c>
-      <c r="C131" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="C131">
+        <v>15970137</v>
       </c>
       <c r="D131" s="1">
-        <v>46140</v>
+        <v>46146</v>
       </c>
       <c r="E131">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132">
-        <v>6640</v>
+        <v>6932</v>
       </c>
       <c r="B132" t="s">
-        <v>12</v>
-      </c>
-      <c r="C132" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="C132">
+        <v>16110881</v>
       </c>
       <c r="D132" s="1">
-        <v>46140</v>
+        <v>46146</v>
       </c>
       <c r="E132">
-        <v>3</v>
+        <v>624</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133">
-        <v>6885</v>
+        <v>6933</v>
       </c>
       <c r="B133" t="s">
-        <v>12</v>
-      </c>
-      <c r="C133" t="s">
-        <v>48</v>
+        <v>15</v>
+      </c>
+      <c r="C133">
+        <v>13991819</v>
       </c>
       <c r="D133" s="1">
-        <v>46140</v>
+        <v>46146</v>
       </c>
       <c r="E133">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134">
-        <v>6831</v>
+        <v>6934</v>
       </c>
       <c r="B134" t="s">
-        <v>12</v>
-      </c>
-      <c r="C134" t="s">
-        <v>31</v>
+        <v>15</v>
+      </c>
+      <c r="C134">
+        <v>14060692</v>
       </c>
       <c r="D134" s="1">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="E134">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135">
-        <v>6906</v>
+        <v>6935</v>
       </c>
       <c r="B135" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C135">
-        <v>15967965</v>
+        <v>13588930</v>
       </c>
       <c r="D135" s="1">
         <v>46146</v>
       </c>
       <c r="E135">
-        <v>39</v>
+        <v>60</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136">
-        <v>6903</v>
+        <v>6936</v>
       </c>
       <c r="B136" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C136">
-        <v>13828817</v>
+        <v>16727617</v>
       </c>
       <c r="D136" s="1">
         <v>46146</v>
       </c>
       <c r="E136">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137">
-        <v>6940</v>
+        <v>6937</v>
       </c>
       <c r="B137" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C137">
-        <v>13833429</v>
+        <v>17800490</v>
       </c>
       <c r="D137" s="1">
         <v>46146</v>
       </c>
       <c r="E137">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138">
-        <v>6939</v>
+        <v>6938</v>
       </c>
       <c r="B138" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C138">
-        <v>11893661</v>
+        <v>14504560</v>
       </c>
       <c r="D138" s="1">
         <v>46146</v>
       </c>
       <c r="E138">
-        <v>72</v>
+        <v>15</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139">
-        <v>6938</v>
+        <v>6939</v>
       </c>
       <c r="B139" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C139">
-        <v>14504560</v>
+        <v>11893661</v>
       </c>
       <c r="D139" s="1">
         <v>46146</v>
       </c>
       <c r="E139">
-        <v>15</v>
+        <v>72</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140">
-        <v>6937</v>
+        <v>6940</v>
       </c>
       <c r="B140" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C140">
-        <v>17800490</v>
+        <v>13833429</v>
       </c>
       <c r="D140" s="1">
         <v>46146</v>
       </c>
       <c r="E140">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141">
-        <v>6936</v>
+        <v>6943</v>
       </c>
       <c r="B141" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C141">
-        <v>16727617</v>
+        <v>14494848</v>
       </c>
       <c r="D141" s="1">
         <v>46146</v>
       </c>
       <c r="E141">
-        <v>50</v>
+        <v>21</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142">
-        <v>6935</v>
+        <v>6944</v>
       </c>
       <c r="B142" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C142">
-        <v>13588930</v>
+        <v>14354620</v>
       </c>
       <c r="D142" s="1">
         <v>46146</v>
       </c>
       <c r="E142">
-        <v>60</v>
+        <v>6</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143">
-        <v>6934</v>
+        <v>6945</v>
       </c>
       <c r="B143" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C143">
-        <v>14060692</v>
+        <v>13991667</v>
       </c>
       <c r="D143" s="1">
         <v>46146</v>
       </c>
       <c r="E143">
-        <v>21</v>
+        <v>33</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144">
-        <v>6933</v>
+        <v>6946</v>
       </c>
       <c r="B144" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C144">
-        <v>13991819</v>
+        <v>17797436</v>
       </c>
       <c r="D144" s="1">
         <v>46146</v>
       </c>
       <c r="E144">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145">
-        <v>6932</v>
+        <v>6947</v>
       </c>
       <c r="B145" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C145">
-        <v>16110881</v>
+        <v>16110422</v>
       </c>
       <c r="D145" s="1">
         <v>46146</v>
       </c>
       <c r="E145">
-        <v>624</v>
+        <v>78</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146">
-        <v>6930</v>
+        <v>6948</v>
       </c>
       <c r="B146" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C146">
-        <v>15970137</v>
+        <v>14496774</v>
       </c>
       <c r="D146" s="1">
         <v>46146</v>
       </c>
       <c r="E146">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147">
-        <v>6929</v>
+        <v>6787</v>
       </c>
       <c r="B147" t="s">
-        <v>22</v>
-      </c>
-      <c r="C147">
-        <v>14153893</v>
+        <v>5</v>
+      </c>
+      <c r="C147" t="s">
+        <v>18</v>
       </c>
       <c r="D147" s="1">
-        <v>46146</v>
+        <v>46147</v>
       </c>
       <c r="E147">
-        <v>57</v>
+        <v>19</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
-        <v>6928</v>
+        <v>6800</v>
       </c>
       <c r="B148" t="s">
-        <v>22</v>
-      </c>
-      <c r="C148">
-        <v>14085079</v>
+        <v>5</v>
+      </c>
+      <c r="C148" t="s">
+        <v>25</v>
       </c>
       <c r="D148" s="1">
-        <v>46146</v>
+        <v>46151</v>
       </c>
       <c r="E148">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149">
-        <v>6914</v>
+        <v>6878</v>
       </c>
       <c r="B149" t="s">
-        <v>22</v>
-      </c>
-      <c r="C149">
-        <v>13832165</v>
+        <v>1</v>
+      </c>
+      <c r="C149" t="s">
+        <v>39</v>
       </c>
       <c r="D149" s="1">
-        <v>46146</v>
+        <v>46151</v>
       </c>
       <c r="E149">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150">
-        <v>6948</v>
+        <v>6548</v>
       </c>
       <c r="B150" t="s">
-        <v>22</v>
-      </c>
-      <c r="C150">
-        <v>14496774</v>
+        <v>1</v>
+      </c>
+      <c r="C150" t="s">
+        <v>4</v>
       </c>
       <c r="D150" s="1">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="E150">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151">
-        <v>6947</v>
+        <v>6555</v>
       </c>
       <c r="B151" t="s">
-        <v>22</v>
-      </c>
-      <c r="C151">
-        <v>16110422</v>
+        <v>1</v>
+      </c>
+      <c r="C151" t="s">
+        <v>3</v>
       </c>
       <c r="D151" s="1">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="E151">
-        <v>78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152">
-        <v>6946</v>
+        <v>6805</v>
       </c>
       <c r="B152" t="s">
-        <v>22</v>
-      </c>
-      <c r="C152">
-        <v>17797436</v>
+        <v>5</v>
+      </c>
+      <c r="C152" t="s">
+        <v>19</v>
       </c>
       <c r="D152" s="1">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="E152">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153">
-        <v>6945</v>
+        <v>6907</v>
       </c>
       <c r="B153" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C153">
-        <v>13991667</v>
+        <v>15967961</v>
       </c>
       <c r="D153" s="1">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="E153">
-        <v>33</v>
+        <v>54</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154">
-        <v>6944</v>
+        <v>6908</v>
       </c>
       <c r="B154" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C154">
-        <v>14354620</v>
+        <v>12864933</v>
       </c>
       <c r="D154" s="1">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="E154">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155">
-        <v>6943</v>
+        <v>6931</v>
       </c>
       <c r="B155" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C155">
-        <v>14494848</v>
+        <v>15970137</v>
       </c>
       <c r="D155" s="1">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="E155">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156">
-        <v>6787</v>
+        <v>6829</v>
       </c>
       <c r="B156" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C156" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D156" s="1">
-        <v>46147</v>
+        <v>46154</v>
       </c>
       <c r="E156">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157">
-        <v>6800</v>
+        <v>6886</v>
       </c>
       <c r="B157" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C157" t="s">
         <v>32</v>
       </c>
       <c r="D157" s="1">
-        <v>46151</v>
+        <v>46155</v>
       </c>
       <c r="E157">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158">
-        <v>6878</v>
+        <v>6890</v>
       </c>
       <c r="B158" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C158" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="D158" s="1">
-        <v>46151</v>
+        <v>46155</v>
       </c>
       <c r="E158">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159">
-        <v>6555</v>
+        <v>6769</v>
       </c>
       <c r="B159" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C159" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D159" s="1">
-        <v>46153</v>
+        <v>46156</v>
       </c>
       <c r="E159">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160">
-        <v>6548</v>
+        <v>6880</v>
       </c>
       <c r="B160" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C160" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="D160" s="1">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -3733,135 +3712,135 @@
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161">
-        <v>6805</v>
+        <v>6881</v>
       </c>
       <c r="B161" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C161" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="D161" s="1">
-        <v>46153</v>
+        <v>46161</v>
       </c>
       <c r="E161">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162">
-        <v>6908</v>
+        <v>6952</v>
       </c>
       <c r="B162" t="s">
-        <v>22</v>
-      </c>
-      <c r="C162">
-        <v>12864933</v>
+        <v>5</v>
+      </c>
+      <c r="C162" t="s">
+        <v>16</v>
       </c>
       <c r="D162" s="1">
-        <v>46153</v>
+        <v>46161</v>
       </c>
       <c r="E162">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163">
-        <v>6907</v>
+        <v>6815</v>
       </c>
       <c r="B163" t="s">
-        <v>22</v>
-      </c>
-      <c r="C163">
-        <v>15967961</v>
+        <v>5</v>
+      </c>
+      <c r="C163" t="s">
+        <v>28</v>
       </c>
       <c r="D163" s="1">
-        <v>46153</v>
+        <v>46163</v>
       </c>
       <c r="E163">
-        <v>54</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164">
-        <v>6931</v>
+        <v>6882</v>
       </c>
       <c r="B164" t="s">
-        <v>22</v>
-      </c>
-      <c r="C164">
-        <v>15970137</v>
+        <v>5</v>
+      </c>
+      <c r="C164" t="s">
+        <v>33</v>
       </c>
       <c r="D164" s="1">
-        <v>46153</v>
+        <v>46165</v>
       </c>
       <c r="E164">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165">
-        <v>6829</v>
+        <v>6905</v>
       </c>
       <c r="B165" t="s">
+        <v>15</v>
+      </c>
+      <c r="C165">
+        <v>13828817</v>
+      </c>
+      <c r="D165" s="1">
+        <v>46167</v>
+      </c>
+      <c r="E165">
         <v>12</v>
-      </c>
-      <c r="C165" t="s">
-        <v>37</v>
-      </c>
-      <c r="D165" s="1">
-        <v>46154</v>
-      </c>
-      <c r="E165">
-        <v>6</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166">
-        <v>6890</v>
+        <v>6915</v>
       </c>
       <c r="B166" t="s">
+        <v>15</v>
+      </c>
+      <c r="C166">
+        <v>13832165</v>
+      </c>
+      <c r="D166" s="1">
+        <v>46167</v>
+      </c>
+      <c r="E166">
         <v>12</v>
-      </c>
-      <c r="C166" t="s">
-        <v>26</v>
-      </c>
-      <c r="D166" s="1">
-        <v>46155</v>
-      </c>
-      <c r="E166">
-        <v>20</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167">
-        <v>6886</v>
+        <v>6806</v>
       </c>
       <c r="B167" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C167" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="D167" s="1">
-        <v>46155</v>
+        <v>46168</v>
       </c>
       <c r="E167">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168">
-        <v>6769</v>
+        <v>6892</v>
       </c>
       <c r="B168" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C168" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D168" s="1">
-        <v>46156</v>
+        <v>46169</v>
       </c>
       <c r="E168">
         <v>15</v>
@@ -3869,254 +3848,254 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169">
-        <v>6880</v>
+        <v>6816</v>
       </c>
       <c r="B169" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C169" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="D169" s="1">
-        <v>46160</v>
+        <v>46170</v>
       </c>
       <c r="E169">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170">
-        <v>6881</v>
+        <v>6888</v>
       </c>
       <c r="B170" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C170" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="D170" s="1">
-        <v>46161</v>
+        <v>46170</v>
       </c>
       <c r="E170">
-        <v>10</v>
+        <v>34</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171">
-        <v>6952</v>
+        <v>6808</v>
       </c>
       <c r="B171" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C171" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D171" s="1">
-        <v>46161</v>
+        <v>46171</v>
       </c>
       <c r="E171">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172">
-        <v>6815</v>
+        <v>6817</v>
       </c>
       <c r="B172" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C172" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D172" s="1">
-        <v>46163</v>
+        <v>46171</v>
       </c>
       <c r="E172">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173">
-        <v>6882</v>
+        <v>6879</v>
       </c>
       <c r="B173" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C173" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="D173" s="1">
-        <v>46165</v>
+        <v>46171</v>
       </c>
       <c r="E173">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174">
-        <v>6905</v>
+        <v>6807</v>
       </c>
       <c r="B174" t="s">
-        <v>22</v>
-      </c>
-      <c r="C174">
-        <v>13828817</v>
+        <v>5</v>
+      </c>
+      <c r="C174" t="s">
+        <v>18</v>
       </c>
       <c r="D174" s="1">
-        <v>46167</v>
+        <v>46175</v>
       </c>
       <c r="E174">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175">
-        <v>6915</v>
+        <v>6904</v>
       </c>
       <c r="B175" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C175">
-        <v>13832165</v>
+        <v>13828817</v>
       </c>
       <c r="D175" s="1">
-        <v>46167</v>
+        <v>46181</v>
       </c>
       <c r="E175">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176">
-        <v>6806</v>
+        <v>6844</v>
       </c>
       <c r="B176" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C176" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D176" s="1">
-        <v>46168</v>
+        <v>46189</v>
       </c>
       <c r="E176">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177">
-        <v>6892</v>
+        <v>6845</v>
       </c>
       <c r="B177" t="s">
+        <v>5</v>
+      </c>
+      <c r="C177" t="s">
         <v>12</v>
       </c>
-      <c r="C177" t="s">
-        <v>18</v>
-      </c>
       <c r="D177" s="1">
-        <v>46169</v>
+        <v>46189</v>
       </c>
       <c r="E177">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178">
-        <v>6816</v>
+        <v>6883</v>
       </c>
       <c r="B178" t="s">
+        <v>5</v>
+      </c>
+      <c r="C178" t="s">
         <v>12</v>
       </c>
-      <c r="C178" t="s">
-        <v>35</v>
-      </c>
       <c r="D178" s="1">
-        <v>46170</v>
+        <v>46196</v>
       </c>
       <c r="E178">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179">
-        <v>6888</v>
+        <v>6884</v>
       </c>
       <c r="B179" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C179" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="D179" s="1">
-        <v>46170</v>
+        <v>46197</v>
       </c>
       <c r="E179">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180">
-        <v>6817</v>
+        <v>6891</v>
       </c>
       <c r="B180" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C180" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="D180" s="1">
-        <v>46171</v>
+        <v>46198</v>
       </c>
       <c r="E180">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181">
-        <v>6808</v>
+        <v>6887</v>
       </c>
       <c r="B181" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C181" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D181" s="1">
-        <v>46171</v>
+        <v>46199</v>
       </c>
       <c r="E181">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182">
-        <v>6879</v>
+        <v>6949</v>
       </c>
       <c r="B182" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="C182" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="D182" s="1">
-        <v>46171</v>
+        <v>46202</v>
       </c>
       <c r="E182">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183">
-        <v>6807</v>
+        <v>6950</v>
       </c>
       <c r="B183" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C183" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D183" s="1">
-        <v>46175</v>
+        <v>46203</v>
       </c>
       <c r="E183">
         <v>9</v>
@@ -4124,194 +4103,45 @@
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184">
-        <v>6904</v>
+        <v>6951</v>
       </c>
       <c r="B184" t="s">
-        <v>22</v>
-      </c>
-      <c r="C184">
-        <v>13828817</v>
+        <v>5</v>
+      </c>
+      <c r="C184" t="s">
+        <v>6</v>
       </c>
       <c r="D184" s="1">
-        <v>46181</v>
+        <v>46203</v>
       </c>
       <c r="E184">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185">
-        <v>6845</v>
+        <v>6889</v>
       </c>
       <c r="B185" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C185" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D185" s="1">
-        <v>46189</v>
+        <v>46228</v>
       </c>
       <c r="E185">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A186">
-        <v>6844</v>
-      </c>
-      <c r="B186" t="s">
-        <v>12</v>
-      </c>
-      <c r="C186" t="s">
-        <v>16</v>
-      </c>
-      <c r="D186" s="1">
-        <v>46189</v>
-      </c>
-      <c r="E186">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A187">
-        <v>6883</v>
-      </c>
-      <c r="B187" t="s">
-        <v>12</v>
-      </c>
-      <c r="C187" t="s">
-        <v>19</v>
-      </c>
-      <c r="D187" s="1">
-        <v>46196</v>
-      </c>
-      <c r="E187">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A188">
-        <v>6884</v>
-      </c>
-      <c r="B188" t="s">
-        <v>12</v>
-      </c>
-      <c r="C188" t="s">
-        <v>49</v>
-      </c>
-      <c r="D188" s="1">
-        <v>46197</v>
-      </c>
-      <c r="E188">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A189">
-        <v>6891</v>
-      </c>
-      <c r="B189" t="s">
-        <v>12</v>
-      </c>
-      <c r="C189" t="s">
-        <v>16</v>
-      </c>
-      <c r="D189" s="1">
-        <v>46198</v>
-      </c>
-      <c r="E189">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A190">
-        <v>6887</v>
-      </c>
-      <c r="B190" t="s">
-        <v>12</v>
-      </c>
-      <c r="C190" t="s">
-        <v>47</v>
-      </c>
-      <c r="D190" s="1">
-        <v>46199</v>
-      </c>
-      <c r="E190">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A191">
-        <v>6949</v>
-      </c>
-      <c r="B191" t="s">
-        <v>12</v>
-      </c>
-      <c r="C191" t="s">
-        <v>19</v>
-      </c>
-      <c r="D191" s="1">
-        <v>46202</v>
-      </c>
-      <c r="E191">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A192">
-        <v>6951</v>
-      </c>
-      <c r="B192" t="s">
-        <v>12</v>
-      </c>
-      <c r="C192" t="s">
-        <v>13</v>
-      </c>
-      <c r="D192" s="1">
-        <v>46203</v>
-      </c>
-      <c r="E192">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A193">
-        <v>6950</v>
-      </c>
-      <c r="B193" t="s">
-        <v>12</v>
-      </c>
-      <c r="C193" t="s">
-        <v>16</v>
-      </c>
-      <c r="D193" s="1">
-        <v>46203</v>
-      </c>
-      <c r="E193">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A194">
-        <v>6889</v>
-      </c>
-      <c r="B194" t="s">
-        <v>12</v>
-      </c>
-      <c r="C194" t="s">
-        <v>45</v>
-      </c>
-      <c r="D194" s="1">
-        <v>46228</v>
-      </c>
-      <c r="E194">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E194" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E218">
+  <autoFilter ref="A1:E185" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E185">
+      <sortCondition ref="D1:D185"/>
+    </sortState>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E209">
     <sortCondition ref="D1"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>